<commit_message>
progress: 60 village workbooks (sivaramans-llin 2026-10-10T15:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Pethikuppam_13.433004_80.120213.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Pethikuppam_13.433004_80.120213.xlsx
@@ -3794,6 +3794,11 @@
           <t>334</t>
         </is>
       </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -3801,6 +3806,11 @@
           <t>335</t>
         </is>
       </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -3808,6 +3818,11 @@
           <t>337</t>
         </is>
       </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -3815,6 +3830,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -3822,6 +3842,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -3829,6 +3854,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3A, 2A3B, 2A4, 2A5, 2A6, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -3836,6 +3866,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -3843,6 +3878,11 @@
           <t>37</t>
         </is>
       </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -3850,6 +3890,11 @@
           <t>38</t>
         </is>
       </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -3857,6 +3902,11 @@
           <t>39</t>
         </is>
       </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -3864,6 +3914,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -3871,6 +3926,11 @@
           <t>40</t>
         </is>
       </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -3878,6 +3938,11 @@
           <t>41</t>
         </is>
       </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -3885,6 +3950,11 @@
           <t>42</t>
         </is>
       </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -3892,6 +3962,11 @@
           <t>43</t>
         </is>
       </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 1C, 1D, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -3899,6 +3974,11 @@
           <t>44</t>
         </is>
       </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -3906,6 +3986,11 @@
           <t>45</t>
         </is>
       </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -3913,6 +3998,11 @@
           <t>46</t>
         </is>
       </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -3920,6 +4010,11 @@
           <t>47</t>
         </is>
       </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -3927,6 +4022,11 @@
           <t>48</t>
         </is>
       </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B1, 5B2</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -3934,6 +4034,11 @@
           <t>49</t>
         </is>
       </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -3941,6 +4046,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4, 5A1, 5A2, 5A3, 5B, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -3948,6 +4058,11 @@
           <t>50</t>
         </is>
       </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -3955,6 +4070,11 @@
           <t>51</t>
         </is>
       </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -3962,6 +4082,11 @@
           <t>52</t>
         </is>
       </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -3969,6 +4094,11 @@
           <t>53</t>
         </is>
       </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -3976,6 +4106,11 @@
           <t>54</t>
         </is>
       </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -3983,6 +4118,11 @@
           <t>55</t>
         </is>
       </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D1, 1D2A, 1D2B, 2A1, 2A2, 2B1, 2B2, 2C1, 2C2, 3A, 3B, 4</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -3990,6 +4130,11 @@
           <t>56</t>
         </is>
       </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -3997,6 +4142,11 @@
           <t>57</t>
         </is>
       </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -4004,6 +4154,11 @@
           <t>58/A</t>
         </is>
       </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -4011,6 +4166,11 @@
           <t>58/B</t>
         </is>
       </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -4018,6 +4178,11 @@
           <t>59</t>
         </is>
       </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -4025,6 +4190,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -4032,6 +4202,11 @@
           <t>60</t>
         </is>
       </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -4039,6 +4214,11 @@
           <t>61</t>
         </is>
       </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -4046,6 +4226,11 @@
           <t>62</t>
         </is>
       </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1A5A, 1A5B, 1B, 2, 3A1, 3A2, 3A3, 3B, 4A, 4B, 4C, 5A1, 5A2, 5A3, 5B</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -4053,6 +4238,11 @@
           <t>63</t>
         </is>
       </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -4060,6 +4250,11 @@
           <t>64</t>
         </is>
       </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>10, 100, 101, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A10, 1A11, 1A12, 1A13, 1A1A1A, 1A2, 1A3, 1A4, 1A5, 1A6, 1A7, 1A8, 1A9, 1B1A1, 1B2, 1B3, 1B4, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1A, 2A1B, 2A1C, 2A2, 2A3, 2B, 30, 31, 32, 33, 34, 35, 36, 37, 38A, 38B, 39, 3A1, 3A2, 3A3, 3B1B1, 3B2, 3B3, 3B4, 3B5A, 3B5B, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 7, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 8, 80, 81, 82, 83, 84, 85, 86, 87, 88, 89, 9, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -4067,6 +4262,11 @@
           <t>65</t>
         </is>
       </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1, 1B2, 1B3, 1B4, 1B5, 2A, 2B, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -4074,6 +4274,11 @@
           <t>66</t>
         </is>
       </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -4081,6 +4286,11 @@
           <t>67</t>
         </is>
       </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A2A, 1C, 2A1A, 2A1B, 2A1C, 2A2, 2B, 2C1, 2C2</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -4088,6 +4298,11 @@
           <t>68</t>
         </is>
       </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -4095,6 +4310,11 @@
           <t>69</t>
         </is>
       </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A3A1A, 1A3A2, 1A3B1, 1A3B2, 1B1, 1B2, 1C1, 1C2, 2A1, 2A2, 2B1A, 2B1B, 2B2, 3A1A, 3A1B, 3A2A1, 3A2A2, 3A2B1, 3A2B2, 3B1, 3B2, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -4102,6 +4322,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>10, 11, 1A1A1, 1A1B, 1A2A1, 1A2B, 1A3, 1B, 1C, 1D, 1E, 2A1, 2A2, 2B, 2C, 3A, 3B, 4A1A1, 4A2, 4A3, 4B1, 4B2, 4B3, 4B4, 5A1A, 5A2A, 5A2B, 5A2C, 5A3, 5B, 5C, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -4109,6 +4334,11 @@
           <t>70</t>
         </is>
       </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -4116,6 +4346,11 @@
           <t>71</t>
         </is>
       </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>1A, 1B, 3, 4A, 4B, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -4123,6 +4358,11 @@
           <t>72</t>
         </is>
       </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -4130,6 +4370,11 @@
           <t>73</t>
         </is>
       </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -4137,6 +4382,11 @@
           <t>74</t>
         </is>
       </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -4144,6 +4394,11 @@
           <t>75</t>
         </is>
       </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>17, 1A, 1B, 1C, 1D, 1E, 1G1, 1G2, 1G3, 1H, 1I, 1J, 1K, 1L, 1M, 1N, 1O, 1P, 1R, 1S, 1T, 1U, 2A1, 2A2, 2B, 3A, 3B, 3C, 4A1, 4A2, 4A3, 4B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -4151,6 +4406,11 @@
           <t>76</t>
         </is>
       </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -4158,6 +4418,11 @@
           <t>77</t>
         </is>
       </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>1A, 1B1, 1B2, 1B3, 1B4, 1B5, 1B6, 1B7, 2</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -4165,6 +4430,11 @@
           <t>78</t>
         </is>
       </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -4172,6 +4442,11 @@
           <t>79</t>
         </is>
       </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -4179,6 +4454,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 2, 3, 4A1, 4A2, 4A3, 4B1, 4B2, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -4186,6 +4466,11 @@
           <t>80</t>
         </is>
       </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -4193,6 +4478,11 @@
           <t>81</t>
         </is>
       </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A2A, 1A2B, 1A3, 1B1, 1B2, 1C1, 1C2, 1C3, 1C4, 1C5, 2, 3A1, 3A2, 3B1A, 3B1A2, 3B1A3, 3B1A4, 3B1A5, 3B2, 3C1A, 3C1B, 3C2, 3D1A, 3D1B, 3D1C, 3D1D, 3D1E, 3D2, 3E, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -4200,6 +4490,11 @@
           <t>82/A</t>
         </is>
       </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -4207,6 +4502,11 @@
           <t>82/B</t>
         </is>
       </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -4214,6 +4514,11 @@
           <t>83</t>
         </is>
       </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 3A1, 3A2, 3B, 3C</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -4221,6 +4526,11 @@
           <t>84</t>
         </is>
       </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12A, 12B, 13, 14A, 14B, 15, 16, 17, 18, 19, 20A, 20B, 21A, 21B, 22A, 22B, 23, 24, 25, 26, 27, 28, 29, 2A1A1, 2A1B, 2A1C, 2A3, 3, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 4, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 5, 50, 51, 57, 58, 59, 6, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 7, 70A, 70B, 71, 72, 73, 74, 75, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -4228,6 +4538,11 @@
           <t>85</t>
         </is>
       </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1A, 2B1B, 2B2</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -4235,6 +4550,11 @@
           <t>86</t>
         </is>
       </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -4242,6 +4562,11 @@
           <t>87/A</t>
         </is>
       </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -4249,11 +4574,21 @@
           <t>87/B</t>
         </is>
       </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
           <t>88</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>